<commit_message>
chore: 同步飞书知识库 2026-10-31 04:36 UTC
</commit_message>
<xml_diff>
--- a/dist/sheets/名词表.xlsx
+++ b/dist/sheets/名词表.xlsx
@@ -849,10 +849,10 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="16"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" max="1" min="1" style="0" width="27.533333333333335"/>
-    <col collapsed="false" customWidth="true" hidden="false" max="2" min="2" style="0" width="27.533333333333335"/>
-    <col collapsed="false" customWidth="true" hidden="false" max="3" min="3" style="0" width="29.4"/>
-    <col collapsed="false" customWidth="true" hidden="false" max="4" min="4" style="0" width="94.06666666666666"/>
+    <col collapsed="false" customWidth="true" hidden="false" max="2" min="2" style="0" width="23.267605633802816"/>
+    <col collapsed="false" customWidth="true" hidden="false" max="3" min="3" style="0" width="24.845070422535212"/>
+    <col collapsed="false" customWidth="true" hidden="false" max="4" min="4" style="0" width="79.49295774647888"/>
+    <col collapsed="false" customWidth="true" hidden="false" max="1" min="1" style="0" width="23.267605633802816"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -883,7 +883,7 @@
         <v>8</v>
       </c>
     </row>
-    <row customHeight="true" ht="20" r="3">
+    <row customHeight="true" ht="16.071428571428573" r="3">
       <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
@@ -1011,7 +1011,7 @@
         <v>42</v>
       </c>
     </row>
-    <row customHeight="true" ht="20" r="13">
+    <row customHeight="true" ht="16.071428571428573" r="13">
       <c r="A13" s="1" t="s">
         <v>43</v>
       </c>
@@ -1125,7 +1125,7 @@
         <v>72</v>
       </c>
     </row>
-    <row customHeight="true" ht="20" r="22">
+    <row customHeight="true" ht="16.071428571428573" r="22">
       <c r="A22" s="1" t="s">
         <v>73</v>
       </c>
@@ -1150,7 +1150,7 @@
         <v>77</v>
       </c>
     </row>
-    <row customHeight="true" ht="20" r="24">
+    <row customHeight="true" ht="16.071428571428573" r="24">
       <c r="A24" s="1" t="s">
         <v>78</v>
       </c>

</xml_diff>